<commit_message>
Atualizar dados e lógica de precedência da ocupação do CD
Co-authored-by: base44-builder[bot] <245833847+base44-builder[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/planilhas/ocupacao-cd.xlsx
+++ b/public/planilhas/ocupacao-cd.xlsx
@@ -1,69 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011" filterPrivacy="true"/>
   <sheets>
-    <sheet sheetId="1" name="Resultado" state="visible" r:id="rId4"/>
+    <sheet name="Resultado" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
-  <si>
-    <t>WF0126 - Ocupação do Centro de Distribuição</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo Relatório: Local de Armazenagem
-Status: Todos
-Lado da Rua: Todos
-Agrupado: Não
-</t>
-  </si>
-  <si>
-    <t>Tipo LA</t>
-  </si>
-  <si>
-    <t>Situação</t>
-  </si>
-  <si>
-    <t>Quantidade</t>
-  </si>
-  <si>
-    <t>PALETE PADRAO (1)</t>
-  </si>
-  <si>
-    <t>Livre</t>
-  </si>
-  <si>
-    <t>Ocupado</t>
-  </si>
-  <si>
-    <t>Bloqueado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  --subtotal--</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ----TOTAL----&gt;</t>
-  </si>
-  <si>
-    <t>Copyright © FullSoft Mobile Solutions - www.fullsoft.com.br</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -86,43 +64,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="table" displayName="table" ref="A3:C8" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A3:C8">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Tipo LA" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="Situação" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Quantidade" totalsRowFunction="none"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -446,96 +396,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="11"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>WF0126 - Ocupação do Centro de Distribuição</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tipo Relatório: Local de Armazenagem_x000d_
+Status: Todos_x000d_
+Lado da Rua: Todos_x000d_
+Agrupado: Não_x000d_
+</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Tipo LA</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Situação</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Quantidade</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PALETE PADRAO (1)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Livre</v>
       </c>
       <c r="C4">
-        <v>1895</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
+        <v>1733</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PALETE PADRAO (1)</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Ocupado</v>
       </c>
       <c r="C5">
-        <v>3685</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
+        <v>3733</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PALETE PADRAO (1)</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Bloqueado</v>
       </c>
       <c r="C6">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>PALETE PADRAO (1)</v>
+      </c>
+      <c r="B7" t="str">
+        <v xml:space="preserve">  --subtotal--</v>
       </c>
       <c r="C7">
-        <v>5735</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>10</v>
+        <v>5557</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="str">
+        <v xml:space="preserve">  ----TOTAL----&gt;</v>
       </c>
       <c r="C8">
-        <v>5735</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
+        <v>5557</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Copyright © FullSoft Mobile Solutions - www.fullsoft.com.br</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -544,12 +488,8 @@
     <mergeCell ref="A9:C9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <headerFooter>
-    <oddFooter>Pág &amp;P de &amp;N</oddFooter>
-  </headerFooter>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>